<commit_message>
books for February voting, fixing issues with the view
</commit_message>
<xml_diff>
--- a/books.xlsx
+++ b/books.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9000"/>
+    <workbookView windowWidth="11520" windowHeight="8280"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -38,148 +38,148 @@
     <t>Cover</t>
   </si>
   <si>
+    <t>This Woven Kingdom</t>
+  </si>
+  <si>
     <t>Taheren Mafi</t>
   </si>
   <si>
-    <t>This Woven Kingdom</t>
-  </si>
-  <si>
     <t>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1634235371i/56554281.jpg</t>
   </si>
   <si>
-    <t>Kylie Snow</t>
-  </si>
-  <si>
-    <t>The Lies of Lena</t>
-  </si>
-  <si>
-    <t>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1708376993i/208884873.jpg</t>
-  </si>
-  <si>
-    <t>Dani Francis</t>
-  </si>
-  <si>
-    <t>Silver Elite</t>
-  </si>
-  <si>
-    <t>https://images-na.ssl-images-amazon.com/images/S/compressed.photo.goodreads.com/books/1728609987i/217245572.jpg</t>
+    <t>Wild Reverence</t>
+  </si>
+  <si>
+    <t>Rebecca Ross</t>
+  </si>
+  <si>
+    <t>https://media.s-bol.com/YL0J0pDW5B4W/KOz0QJx/767x1200.jpg</t>
+  </si>
+  <si>
+    <t>The Bloody Branch</t>
+  </si>
+  <si>
+    <t>Brigid Lowe</t>
+  </si>
+  <si>
+    <t>https://cdn.penguin.co.uk/dam-assets/books/9781787305250/9781787305250-jacket-large.jpg</t>
+  </si>
+  <si>
+    <t>The Serpent and the Wolf</t>
   </si>
   <si>
     <t>Rebecca Robinson</t>
   </si>
   <si>
-    <t>The Serpent and the Wolf</t>
-  </si>
-  <si>
     <t>https://m.media-amazon.com/images/I/7186YNOq9wL._SY466_.jpg</t>
   </si>
   <si>
+    <t>Shield of Sparrows</t>
+  </si>
+  <si>
     <t>Devney Perry</t>
   </si>
   <si>
-    <t>Shield of Sparrows</t>
-  </si>
-  <si>
     <t>https://devneyperry.com/wp-content/uploads/2024/11/ShieldOfSparrows-1600-1.jpg</t>
   </si>
   <si>
-    <t>Brandon Sanderson</t>
-  </si>
-  <si>
-    <t>Mistborn: The Final Empire</t>
-  </si>
-  <si>
-    <t>https://cdn.kobo.com/book-images/262e58e4-8ab1-4ab4-b89a-eac880b1a0a1/1200/1200/False/mistborn.jpg</t>
+    <t>A Fate Forged in Fire</t>
   </si>
   <si>
     <t>Hazel McBride</t>
   </si>
   <si>
-    <t>A Fate Forged in Fire</t>
-  </si>
-  <si>
     <t>https://m.media-amazon.com/images/I/91E0OEUccOL._UF1000,1000_QL80_.jpg</t>
   </si>
   <si>
+    <t>City of Stairs</t>
+  </si>
+  <si>
     <t>R. J. Bennett</t>
   </si>
   <si>
-    <t>City of Stairs</t>
-  </si>
-  <si>
     <t>https://media.s-bol.com/JkE8nB1gOpr9/mZ8qPNp/546x840.jpg</t>
   </si>
   <si>
+    <t>Red Rising</t>
+  </si>
+  <si>
     <t>Pierce Brown</t>
   </si>
   <si>
-    <t>Red Rising</t>
-  </si>
-  <si>
     <t>https://m.media-amazon.com/images/I/81YOu17CxTL._UF1000,1000_QL80_.jpg</t>
   </si>
   <si>
+    <t>The Second Death of Locke</t>
+  </si>
+  <si>
     <t>V. L. Bovalino</t>
   </si>
   <si>
-    <t>The Second Death of Locke</t>
-  </si>
-  <si>
     <t>https://m.media-amazon.com/images/I/81XCo+49lBL._AC_UF894,1000_QL80_.jpg</t>
   </si>
   <si>
+    <t>Masters of Death</t>
+  </si>
+  <si>
     <t>Olivie Blake</t>
   </si>
   <si>
-    <t>Masters of Death</t>
-  </si>
-  <si>
     <t>https://m.media-amazon.com/images/I/81MKKCAmRgL._AC_UF894,1000_QL80_.jpg</t>
   </si>
   <si>
-    <t>Invi Wright</t>
-  </si>
-  <si>
-    <t>The Female</t>
-  </si>
-  <si>
-    <t>https://api.bruna.nl/images/active/carrousel/fullsize/9781966285007_front.jpg</t>
-  </si>
-  <si>
-    <t>Ali Hazelwood</t>
-  </si>
-  <si>
-    <t>Bride</t>
-  </si>
-  <si>
-    <t>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1730451646i/181344829.jpg</t>
-  </si>
-  <si>
-    <t>Erin Sterling</t>
-  </si>
-  <si>
-    <t>The Ex Hex</t>
-  </si>
-  <si>
-    <t>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1619305366i/56554626.jpg</t>
-  </si>
-  <si>
-    <t>RuNyx</t>
-  </si>
-  <si>
-    <t>Enigma</t>
-  </si>
-  <si>
-    <t>https://mpd-biblio-covers.imgix.net/9781250334244.jpg?w=300&amp;dpr=3</t>
+    <t>The Fifth Season</t>
+  </si>
+  <si>
+    <t>N. K. Jemisin</t>
+  </si>
+  <si>
+    <t>https://en.wikipedia.org/wiki/The_Fifth_Season_%28novel%29#/media/File%3AThe_Fifth_Season_(novel).jpg</t>
+  </si>
+  <si>
+    <t>The Wolf King</t>
+  </si>
+  <si>
+    <t>Lauren Palphreyman</t>
+  </si>
+  <si>
+    <t>https://media.s-bol.com/KqEy5EnjP52J/58KrVGX/780x1200.jpg</t>
+  </si>
+  <si>
+    <t>Smoke and Scar</t>
+  </si>
+  <si>
+    <t>Gretchen Powell</t>
+  </si>
+  <si>
+    <t>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1735223143i/221866459.jpg</t>
+  </si>
+  <si>
+    <t>Tusk Love</t>
   </si>
   <si>
     <t>Thea Guanzon</t>
   </si>
   <si>
-    <t>Tusk Love</t>
-  </si>
-  <si>
     <t>https://i0.wp.com/thenerddaily.com/wp-content/uploads/2025/07/Tusk-Love-by-Thea-Guanzon.jpg?w=964&amp;ssl=1</t>
+  </si>
+  <si>
+    <t>Son of the morning</t>
+  </si>
+  <si>
+    <t>Awaeke Emezi</t>
+  </si>
+  <si>
+    <t>https://media.s-bol.com/7ZEXzNWR9llj/mwjmkQr/546x840.jpg</t>
+  </si>
+  <si>
+    <t>the adventures of Amin al-sirafi</t>
+  </si>
+  <si>
+    <t>S A Chakraborty</t>
+  </si>
+  <si>
+    <t>https://encrypted-tbn0.gstatic.com/images?q=tbn:ANd9GcTaGkpCJ9Yc_EYLHWdv-FxadI9qyYSCvpB_G57XxblwTw&amp;s=10</t>
   </si>
 </sst>
 </file>
@@ -192,7 +192,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="25">
+  <fonts count="24">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -228,12 +228,6 @@
       <charset val="134"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color rgb="FF1E1915"/>
-      <name val="Copernicus"/>
-      <charset val="134"/>
-    </font>
-    <font>
       <u/>
       <sz val="11"/>
       <color rgb="FF0000FF"/>
@@ -378,7 +372,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="34">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -388,6 +382,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -719,137 +719,137 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="22" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -865,7 +865,16 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1" readingOrder="1"/>
     </xf>
   </cellXfs>
@@ -1431,25 +1440,25 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" ht="53.55" spans="1:3">
-      <c r="A3" s="2" t="s">
+    <row r="3" ht="40.35" spans="1:3">
+      <c r="A3" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="5" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" ht="53.55" spans="1:3">
+    <row r="4" ht="40.35" spans="1:3">
       <c r="A4" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="5" t="s">
         <v>11</v>
       </c>
     </row>
@@ -1475,7 +1484,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" ht="53.55" spans="1:3">
+    <row r="7" ht="40.35" spans="1:3">
       <c r="A7" s="2" t="s">
         <v>18</v>
       </c>
@@ -1541,14 +1550,14 @@
         <v>35</v>
       </c>
     </row>
-    <row r="13" ht="27.15" spans="1:3">
+    <row r="13" ht="40.35" spans="1:3">
       <c r="A13" s="2" t="s">
         <v>36</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="5" t="s">
         <v>38</v>
       </c>
     </row>
@@ -1563,14 +1572,14 @@
         <v>41</v>
       </c>
     </row>
-    <row r="15" ht="53.55" spans="1:3">
+    <row r="15" ht="40.35" spans="1:3">
       <c r="A15" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C15" s="6" t="s">
         <v>44</v>
       </c>
     </row>
@@ -1585,7 +1594,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="17" ht="40.35" spans="1:3">
+    <row r="17" ht="53.55" spans="1:3">
       <c r="A17" s="2" t="s">
         <v>48</v>
       </c>
@@ -1597,25 +1606,28 @@
       </c>
     </row>
     <row r="18" ht="15.15" spans="1:3">
-      <c r="A18" s="2"/>
-      <c r="B18" s="2"/>
-      <c r="C18" s="3"/>
+      <c r="A18" s="7"/>
+      <c r="B18" s="7"/>
+      <c r="C18" s="8"/>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="C2" r:id="rId1" display="https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1634235371i/56554281.jpg" tooltip="https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1634235371i/56554281.jpg"/>
-    <hyperlink ref="C4" r:id="rId2" display="https://images-na.ssl-images-amazon.com/images/S/compressed.photo.goodreads.com/books/1728609987i/217245572.jpg" tooltip="https://images-na.ssl-images-amazon.com/images/S/compressed.photo.goodreads.com/books/1728609987i/217245572.jpg"/>
-    <hyperlink ref="C5" r:id="rId3" display="https://m.media-amazon.com/images/I/7186YNOq9wL._SY466_.jpg" tooltip="https://m.media-amazon.com/images/I/7186YNOq9wL._SY466_.jpg"/>
-    <hyperlink ref="C6" r:id="rId4" display="https://devneyperry.com/wp-content/uploads/2024/11/ShieldOfSparrows-1600-1.jpg" tooltip="https://devneyperry.com/wp-content/uploads/2024/11/ShieldOfSparrows-1600-1.jpg"/>
-    <hyperlink ref="C7" r:id="rId5" display="https://cdn.kobo.com/book-images/262e58e4-8ab1-4ab4-b89a-eac880b1a0a1/1200/1200/False/mistborn.jpg" tooltip="https://cdn.kobo.com/book-images/262e58e4-8ab1-4ab4-b89a-eac880b1a0a1/1200/1200/False/mistborn.jpg"/>
-    <hyperlink ref="C8" r:id="rId6" display="https://m.media-amazon.com/images/I/91E0OEUccOL._UF1000,1000_QL80_.jpg" tooltip="https://m.media-amazon.com/images/I/91E0OEUccOL._UF1000,1000_QL80_.jpg"/>
-    <hyperlink ref="C9" r:id="rId7" display="https://media.s-bol.com/JkE8nB1gOpr9/mZ8qPNp/546x840.jpg" tooltip="https://media.s-bol.com/JkE8nB1gOpr9/mZ8qPNp/546x840.jpg"/>
-    <hyperlink ref="C10" r:id="rId8" display="https://m.media-amazon.com/images/I/81YOu17CxTL._UF1000,1000_QL80_.jpg" tooltip="https://m.media-amazon.com/images/I/81YOu17CxTL._UF1000,1000_QL80_.jpg"/>
-    <hyperlink ref="C11" r:id="rId9" display="https://m.media-amazon.com/images/I/81XCo+49lBL._AC_UF894,1000_QL80_.jpg" tooltip="https://m.media-amazon.com/images/I/81XCo+49lBL._AC_UF894,1000_QL80_.jpg"/>
-    <hyperlink ref="C12" r:id="rId10" display="https://m.media-amazon.com/images/I/81MKKCAmRgL._AC_UF894,1000_QL80_.jpg" tooltip="https://m.media-amazon.com/images/I/81MKKCAmRgL._AC_UF894,1000_QL80_.jpg"/>
-    <hyperlink ref="C13" r:id="rId11" display="https://api.bruna.nl/images/active/carrousel/fullsize/9781966285007_front.jpg" tooltip="https://api.bruna.nl/images/active/carrousel/fullsize/9781966285007_front.jpg"/>
-    <hyperlink ref="C16" r:id="rId12" display="https://mpd-biblio-covers.imgix.net/9781250334244.jpg?w=300&amp;dpr=3" tooltip="https://mpd-biblio-covers.imgix.net/9781250334244.jpg?w=300&amp;dpr=3"/>
-    <hyperlink ref="C17" r:id="rId13" display="https://i0.wp.com/thenerddaily.com/wp-content/uploads/2025/07/Tusk-Love-by-Thea-Guanzon.jpg?w=964&amp;ssl=1" tooltip="https://i0.wp.com/thenerddaily.com/wp-content/uploads/2025/07/Tusk-Love-by-Thea-Guanzon.jpg?w=964&amp;ssl=1"/>
+    <hyperlink ref="C3" r:id="rId2" display="https://media.s-bol.com/YL0J0pDW5B4W/KOz0QJx/767x1200.jpg" tooltip="https://media.s-bol.com/YL0J0pDW5B4W/KOz0QJx/767x1200.jpg"/>
+    <hyperlink ref="C4" r:id="rId3" display="https://cdn.penguin.co.uk/dam-assets/books/9781787305250/9781787305250-jacket-large.jpg" tooltip="https://cdn.penguin.co.uk/dam-assets/books/9781787305250/9781787305250-jacket-large.jpg"/>
+    <hyperlink ref="C5" r:id="rId4" display="https://m.media-amazon.com/images/I/7186YNOq9wL._SY466_.jpg" tooltip="https://m.media-amazon.com/images/I/7186YNOq9wL._SY466_.jpg"/>
+    <hyperlink ref="C6" r:id="rId5" display="https://devneyperry.com/wp-content/uploads/2024/11/ShieldOfSparrows-1600-1.jpg" tooltip="https://devneyperry.com/wp-content/uploads/2024/11/ShieldOfSparrows-1600-1.jpg"/>
+    <hyperlink ref="C7" r:id="rId6" display="https://m.media-amazon.com/images/I/91E0OEUccOL._UF1000,1000_QL80_.jpg" tooltip="https://m.media-amazon.com/images/I/91E0OEUccOL._UF1000,1000_QL80_.jpg"/>
+    <hyperlink ref="C8" r:id="rId7" display="https://media.s-bol.com/JkE8nB1gOpr9/mZ8qPNp/546x840.jpg" tooltip="https://media.s-bol.com/JkE8nB1gOpr9/mZ8qPNp/546x840.jpg"/>
+    <hyperlink ref="C9" r:id="rId8" display="https://m.media-amazon.com/images/I/81YOu17CxTL._UF1000,1000_QL80_.jpg" tooltip="https://m.media-amazon.com/images/I/81YOu17CxTL._UF1000,1000_QL80_.jpg"/>
+    <hyperlink ref="C10" r:id="rId9" display="https://m.media-amazon.com/images/I/81XCo+49lBL._AC_UF894,1000_QL80_.jpg" tooltip="https://m.media-amazon.com/images/I/81XCo+49lBL._AC_UF894,1000_QL80_.jpg"/>
+    <hyperlink ref="C11" r:id="rId10" display="https://m.media-amazon.com/images/I/81MKKCAmRgL._AC_UF894,1000_QL80_.jpg" tooltip="https://m.media-amazon.com/images/I/81MKKCAmRgL._AC_UF894,1000_QL80_.jpg"/>
+    <hyperlink ref="C12" r:id="rId11" display="https://en.wikipedia.org/wiki/The_Fifth_Season_%28novel%29#/media/File%3AThe_Fifth_Season_(novel).jpg"/>
+    <hyperlink ref="C13" r:id="rId12" display="https://media.s-bol.com/KqEy5EnjP52J/58KrVGX/780x1200.jpg" tooltip="https://media.s-bol.com/KqEy5EnjP52J/58KrVGX/780x1200.jpg"/>
+    <hyperlink ref="C14" r:id="rId13" display="https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1735223143i/221866459.jpg" tooltip="https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1735223143i/221866459.jpg"/>
+    <hyperlink ref="C15" r:id="rId14" display="https://i0.wp.com/thenerddaily.com/wp-content/uploads/2025/07/Tusk-Love-by-Thea-Guanzon.jpg?w=964&amp;ssl=1" tooltip="https://i0.wp.com/thenerddaily.com/wp-content/uploads/2025/07/Tusk-Love-by-Thea-Guanzon.jpg?w=964&amp;ssl=1"/>
+    <hyperlink ref="C16" r:id="rId15" display="https://media.s-bol.com/7ZEXzNWR9llj/mwjmkQr/546x840.jpg" tooltip="https://media.s-bol.com/7ZEXzNWR9llj/mwjmkQr/546x840.jpg"/>
+    <hyperlink ref="C17" r:id="rId16" display="https://encrypted-tbn0.gstatic.com/images?q=tbn:ANd9GcTaGkpCJ9Yc_EYLHWdv-FxadI9qyYSCvpB_G57XxblwTw&amp;s=10" tooltip="https://encrypted-tbn0.gstatic.com/images?q=tbn:ANd9GcTaGkpCJ9Yc_EYLHWdv-FxadI9qyYSCvpB_G57XxblwTw&amp;s=10"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>

<commit_message>
books for March voting
</commit_message>
<xml_diff>
--- a/books.xlsx
+++ b/books.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="11520" windowHeight="8280"/>
+    <workbookView windowWidth="23040" windowHeight="8280"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -65,49 +65,40 @@
     <t>https://cdn.penguin.co.uk/dam-assets/books/9781787305250/9781787305250-jacket-large.jpg</t>
   </si>
   <si>
-    <t>The Serpent and the Wolf</t>
-  </si>
-  <si>
-    <t>Rebecca Robinson</t>
-  </si>
-  <si>
-    <t>https://m.media-amazon.com/images/I/7186YNOq9wL._SY466_.jpg</t>
-  </si>
-  <si>
-    <t>Shield of Sparrows</t>
-  </si>
-  <si>
-    <t>Devney Perry</t>
-  </si>
-  <si>
-    <t>https://devneyperry.com/wp-content/uploads/2024/11/ShieldOfSparrows-1600-1.jpg</t>
-  </si>
-  <si>
-    <t>A Fate Forged in Fire</t>
-  </si>
-  <si>
-    <t>Hazel McBride</t>
-  </si>
-  <si>
-    <t>https://m.media-amazon.com/images/I/91E0OEUccOL._UF1000,1000_QL80_.jpg</t>
-  </si>
-  <si>
-    <t>City of Stairs</t>
-  </si>
-  <si>
-    <t>R. J. Bennett</t>
-  </si>
-  <si>
-    <t>https://media.s-bol.com/JkE8nB1gOpr9/mZ8qPNp/546x840.jpg</t>
-  </si>
-  <si>
-    <t>Red Rising</t>
-  </si>
-  <si>
-    <t>Pierce Brown</t>
-  </si>
-  <si>
-    <t>https://m.media-amazon.com/images/I/81YOu17CxTL._UF1000,1000_QL80_.jpg</t>
+    <t>Jade Fire Gold</t>
+  </si>
+  <si>
+    <t>June CL Tan</t>
+  </si>
+  <si>
+    <t>https://images.squarespace-cdn.com/content/v1/5fa4660bb109d3087785cca0/27525d3a-e30b-4d08-ae30-719f400c4a0e/JFG_OC.jpg</t>
+  </si>
+  <si>
+    <t>His Majesty's Dragon</t>
+  </si>
+  <si>
+    <t>Naomi Novik</t>
+  </si>
+  <si>
+    <t>https://upload.wikimedia.org/wikipedia/en/e/e2/Hmsdragon.jpg</t>
+  </si>
+  <si>
+    <t>The Tainted Cup</t>
+  </si>
+  <si>
+    <t>Robert Jackson Bennet</t>
+  </si>
+  <si>
+    <t>https://m.media-amazon.com/images/I/817taI05uEL._AC_UF894,1000_QL80_.jpg</t>
+  </si>
+  <si>
+    <t>The Everlasting</t>
+  </si>
+  <si>
+    <t>Alix E. Harrow</t>
+  </si>
+  <si>
+    <t>https://ik.imagekit.io/panmac/tr:f-auto,di-placeholder_portrait_aMjPtD9YZ.jpg,w-270/edition/9781529061185.jpg</t>
   </si>
   <si>
     <t>The Second Death of Locke</t>
@@ -134,7 +125,7 @@
     <t>N. K. Jemisin</t>
   </si>
   <si>
-    <t>https://en.wikipedia.org/wiki/The_Fifth_Season_%28novel%29#/media/File%3AThe_Fifth_Season_(novel).jpg</t>
+    <t>https://nkjemisin.com/wp-content/uploads/2013/09/Jemisin_FifthSeason-TP.jpg</t>
   </si>
   <si>
     <t>The Wolf King</t>
@@ -155,15 +146,6 @@
     <t>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1735223143i/221866459.jpg</t>
   </si>
   <si>
-    <t>Tusk Love</t>
-  </si>
-  <si>
-    <t>Thea Guanzon</t>
-  </si>
-  <si>
-    <t>https://i0.wp.com/thenerddaily.com/wp-content/uploads/2025/07/Tusk-Love-by-Thea-Guanzon.jpg?w=964&amp;ssl=1</t>
-  </si>
-  <si>
     <t>Son of the morning</t>
   </si>
   <si>
@@ -173,13 +155,31 @@
     <t>https://media.s-bol.com/7ZEXzNWR9llj/mwjmkQr/546x840.jpg</t>
   </si>
   <si>
-    <t>the adventures of Amin al-sirafi</t>
+    <t>The Adventures of Amina Al-Sirafi</t>
   </si>
   <si>
     <t>S A Chakraborty</t>
   </si>
   <si>
     <t>https://encrypted-tbn0.gstatic.com/images?q=tbn:ANd9GcTaGkpCJ9Yc_EYLHWdv-FxadI9qyYSCvpB_G57XxblwTw&amp;s=10</t>
+  </si>
+  <si>
+    <t>The Scattered Bones</t>
+  </si>
+  <si>
+    <t>Nicole Scarano</t>
+  </si>
+  <si>
+    <t>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1692132539i/162728103.jpg</t>
+  </si>
+  <si>
+    <t>A Fate Inked in Blood</t>
+  </si>
+  <si>
+    <t>Danielle L. Jensen</t>
+  </si>
+  <si>
+    <t>https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1690490514i/165940202.jpg</t>
   </si>
 </sst>
 </file>
@@ -849,7 +849,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -866,15 +866,6 @@
       <alignment wrapText="1" readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1" readingOrder="1"/>
     </xf>
   </cellXfs>
@@ -1410,7 +1401,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="2"/>
   <cols>
     <col min="1" max="1" width="34.7777777777778" customWidth="1"/>
@@ -1462,7 +1453,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" ht="40.35" spans="1:3">
+    <row r="5" ht="53.55" spans="1:3">
       <c r="A5" s="2" t="s">
         <v>12</v>
       </c>
@@ -1473,7 +1464,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" ht="40.35" spans="1:3">
+    <row r="6" ht="27.15" spans="1:3">
       <c r="A6" s="2" t="s">
         <v>15</v>
       </c>
@@ -1495,7 +1486,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" ht="40.35" spans="1:3">
+    <row r="8" ht="53.55" spans="1:3">
       <c r="A8" s="2" t="s">
         <v>21</v>
       </c>
@@ -1535,7 +1526,7 @@
       <c r="B11" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C11" s="5" t="s">
         <v>32</v>
       </c>
     </row>
@@ -1546,22 +1537,22 @@
       <c r="B12" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="5" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="13" ht="40.35" spans="1:3">
+    <row r="13" ht="53.55" spans="1:3">
       <c r="A13" s="2" t="s">
         <v>36</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="C13" s="3" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="14" ht="53.55" spans="1:3">
+    <row r="14" ht="40.35" spans="1:3">
       <c r="A14" s="2" t="s">
         <v>39</v>
       </c>
@@ -1572,18 +1563,18 @@
         <v>41</v>
       </c>
     </row>
-    <row r="15" ht="40.35" spans="1:3">
+    <row r="15" ht="53.55" spans="1:3">
       <c r="A15" s="2" t="s">
         <v>42</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="C15" s="6" t="s">
+      <c r="C15" s="3" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="16" ht="40.35" spans="1:3">
+    <row r="16" ht="53.55" spans="1:3">
       <c r="A16" s="2" t="s">
         <v>45</v>
       </c>
@@ -1604,30 +1595,25 @@
       <c r="C17" s="3" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="18" ht="15.15" spans="1:3">
-      <c r="A18" s="7"/>
-      <c r="B18" s="7"/>
-      <c r="C18" s="8"/>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="C2" r:id="rId1" display="https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1634235371i/56554281.jpg" tooltip="https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1634235371i/56554281.jpg"/>
     <hyperlink ref="C3" r:id="rId2" display="https://media.s-bol.com/YL0J0pDW5B4W/KOz0QJx/767x1200.jpg" tooltip="https://media.s-bol.com/YL0J0pDW5B4W/KOz0QJx/767x1200.jpg"/>
     <hyperlink ref="C4" r:id="rId3" display="https://cdn.penguin.co.uk/dam-assets/books/9781787305250/9781787305250-jacket-large.jpg" tooltip="https://cdn.penguin.co.uk/dam-assets/books/9781787305250/9781787305250-jacket-large.jpg"/>
-    <hyperlink ref="C5" r:id="rId4" display="https://m.media-amazon.com/images/I/7186YNOq9wL._SY466_.jpg" tooltip="https://m.media-amazon.com/images/I/7186YNOq9wL._SY466_.jpg"/>
-    <hyperlink ref="C6" r:id="rId5" display="https://devneyperry.com/wp-content/uploads/2024/11/ShieldOfSparrows-1600-1.jpg" tooltip="https://devneyperry.com/wp-content/uploads/2024/11/ShieldOfSparrows-1600-1.jpg"/>
-    <hyperlink ref="C7" r:id="rId6" display="https://m.media-amazon.com/images/I/91E0OEUccOL._UF1000,1000_QL80_.jpg" tooltip="https://m.media-amazon.com/images/I/91E0OEUccOL._UF1000,1000_QL80_.jpg"/>
-    <hyperlink ref="C8" r:id="rId7" display="https://media.s-bol.com/JkE8nB1gOpr9/mZ8qPNp/546x840.jpg" tooltip="https://media.s-bol.com/JkE8nB1gOpr9/mZ8qPNp/546x840.jpg"/>
-    <hyperlink ref="C9" r:id="rId8" display="https://m.media-amazon.com/images/I/81YOu17CxTL._UF1000,1000_QL80_.jpg" tooltip="https://m.media-amazon.com/images/I/81YOu17CxTL._UF1000,1000_QL80_.jpg"/>
-    <hyperlink ref="C10" r:id="rId9" display="https://m.media-amazon.com/images/I/81XCo+49lBL._AC_UF894,1000_QL80_.jpg" tooltip="https://m.media-amazon.com/images/I/81XCo+49lBL._AC_UF894,1000_QL80_.jpg"/>
-    <hyperlink ref="C11" r:id="rId10" display="https://m.media-amazon.com/images/I/81MKKCAmRgL._AC_UF894,1000_QL80_.jpg" tooltip="https://m.media-amazon.com/images/I/81MKKCAmRgL._AC_UF894,1000_QL80_.jpg"/>
-    <hyperlink ref="C12" r:id="rId11" display="https://en.wikipedia.org/wiki/The_Fifth_Season_%28novel%29#/media/File%3AThe_Fifth_Season_(novel).jpg"/>
-    <hyperlink ref="C13" r:id="rId12" display="https://media.s-bol.com/KqEy5EnjP52J/58KrVGX/780x1200.jpg" tooltip="https://media.s-bol.com/KqEy5EnjP52J/58KrVGX/780x1200.jpg"/>
-    <hyperlink ref="C14" r:id="rId13" display="https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1735223143i/221866459.jpg" tooltip="https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1735223143i/221866459.jpg"/>
-    <hyperlink ref="C15" r:id="rId14" display="https://i0.wp.com/thenerddaily.com/wp-content/uploads/2025/07/Tusk-Love-by-Thea-Guanzon.jpg?w=964&amp;ssl=1" tooltip="https://i0.wp.com/thenerddaily.com/wp-content/uploads/2025/07/Tusk-Love-by-Thea-Guanzon.jpg?w=964&amp;ssl=1"/>
-    <hyperlink ref="C16" r:id="rId15" display="https://media.s-bol.com/7ZEXzNWR9llj/mwjmkQr/546x840.jpg" tooltip="https://media.s-bol.com/7ZEXzNWR9llj/mwjmkQr/546x840.jpg"/>
-    <hyperlink ref="C17" r:id="rId16" display="https://encrypted-tbn0.gstatic.com/images?q=tbn:ANd9GcTaGkpCJ9Yc_EYLHWdv-FxadI9qyYSCvpB_G57XxblwTw&amp;s=10" tooltip="https://encrypted-tbn0.gstatic.com/images?q=tbn:ANd9GcTaGkpCJ9Yc_EYLHWdv-FxadI9qyYSCvpB_G57XxblwTw&amp;s=10"/>
+    <hyperlink ref="C5" r:id="rId4" display="https://images.squarespace-cdn.com/content/v1/5fa4660bb109d3087785cca0/27525d3a-e30b-4d08-ae30-719f400c4a0e/JFG_OC.jpg" tooltip="https://images.squarespace-cdn.com/content/v1/5fa4660bb109d3087785cca0/27525d3a-e30b-4d08-ae30-719f400c4a0e/JFG_OC.jpg"/>
+    <hyperlink ref="C6" r:id="rId5" display="https://upload.wikimedia.org/wikipedia/en/e/e2/Hmsdragon.jpg" tooltip="https://upload.wikimedia.org/wikipedia/en/e/e2/Hmsdragon.jpg"/>
+    <hyperlink ref="C7" r:id="rId6" display="https://m.media-amazon.com/images/I/817taI05uEL._AC_UF894,1000_QL80_.jpg" tooltip="https://m.media-amazon.com/images/I/817taI05uEL._AC_UF894,1000_QL80_.jpg"/>
+    <hyperlink ref="C8" r:id="rId7" display="https://ik.imagekit.io/panmac/tr:f-auto,di-placeholder_portrait_aMjPtD9YZ.jpg,w-270/edition/9781529061185.jpg" tooltip="https://ik.imagekit.io/panmac/tr:f-auto,di-placeholder_portrait_aMjPtD9YZ.jpg,w-270/edition/9781529061185.jpg"/>
+    <hyperlink ref="C9" r:id="rId8" display="https://m.media-amazon.com/images/I/81XCo+49lBL._AC_UF894,1000_QL80_.jpg" tooltip="https://m.media-amazon.com/images/I/81XCo+49lBL._AC_UF894,1000_QL80_.jpg"/>
+    <hyperlink ref="C10" r:id="rId9" display="https://m.media-amazon.com/images/I/81MKKCAmRgL._AC_UF894,1000_QL80_.jpg" tooltip="https://m.media-amazon.com/images/I/81MKKCAmRgL._AC_UF894,1000_QL80_.jpg"/>
+    <hyperlink ref="C11" r:id="rId10" display="https://nkjemisin.com/wp-content/uploads/2013/09/Jemisin_FifthSeason-TP.jpg" tooltip="https://nkjemisin.com/wp-content/uploads/2013/09/Jemisin_FifthSeason-TP.jpg"/>
+    <hyperlink ref="C12" r:id="rId11" display="https://media.s-bol.com/KqEy5EnjP52J/58KrVGX/780x1200.jpg" tooltip="https://media.s-bol.com/KqEy5EnjP52J/58KrVGX/780x1200.jpg"/>
+    <hyperlink ref="C13" r:id="rId12" display="https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1735223143i/221866459.jpg" tooltip="https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1735223143i/221866459.jpg"/>
+    <hyperlink ref="C14" r:id="rId13" display="https://media.s-bol.com/7ZEXzNWR9llj/mwjmkQr/546x840.jpg" tooltip="https://media.s-bol.com/7ZEXzNWR9llj/mwjmkQr/546x840.jpg"/>
+    <hyperlink ref="C15" r:id="rId14" display="https://encrypted-tbn0.gstatic.com/images?q=tbn:ANd9GcTaGkpCJ9Yc_EYLHWdv-FxadI9qyYSCvpB_G57XxblwTw&amp;s=10" tooltip="https://encrypted-tbn0.gstatic.com/images?q=tbn:ANd9GcTaGkpCJ9Yc_EYLHWdv-FxadI9qyYSCvpB_G57XxblwTw&amp;s=10"/>
+    <hyperlink ref="C16" r:id="rId15" display="https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1692132539i/162728103.jpg" tooltip="https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1692132539i/162728103.jpg"/>
+    <hyperlink ref="C17" r:id="rId16" display="https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1690490514i/165940202.jpg" tooltip="https://m.media-amazon.com/images/S/compressed.photo.goodreads.com/books/1690490514i/165940202.jpg"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>